<commit_message>
Intermediate: Implemented cache for HasherEventMap
</commit_message>
<xml_diff>
--- a/android/devHelpers/DataClassHelper.xlsx
+++ b/android/devHelpers/DataClassHelper.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jameswhite/Projects/flutter/HC/HarrierCentral/HarrierCentralMobile-Flutter/android/devHelpers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8C12A0-180E-F643-9956-17DDAAE066D4}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E195015F-4387-644F-853A-B2CCED30F208}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="20540" xr2:uid="{50A37692-8663-7F4C-91F6-2AE3BA380A00}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="23">
   <si>
     <t>wireName</t>
   </si>
@@ -68,16 +68,16 @@
   </si>
   <si>
     <r>
-      <t>coalesce</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
+      <t xml:space="preserve">[id] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Consolas"/>
+        <family val="2"/>
+      </rPr>
+      <t>as</t>
     </r>
     <r>
       <rPr>
@@ -86,16 +86,12 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t>h</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
+      <t xml:space="preserve"> hemId</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>,</t>
     </r>
     <r>
       <rPr>
@@ -104,43 +100,39 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t>FirstName</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
+      <t xml:space="preserve">[UserId] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Consolas"/>
+        <family val="2"/>
+      </rPr>
+      <t>as</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Consolas"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> userId</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>,</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>''</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
         <color theme="1"/>
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> </t>
+      <t xml:space="preserve">[EventId] </t>
     </r>
     <r>
       <rPr>
@@ -158,31 +150,13 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> firstName</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
+      <t xml:space="preserve"> eventId</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>,</t>
     </r>
-  </si>
-  <si>
-    <r>
-      <t>coalesce</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
     <r>
       <rPr>
         <sz val="10"/>
@@ -190,16 +164,16 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t>h</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
+      <t xml:space="preserve">[UserStartEvent] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Consolas"/>
+        <family val="2"/>
+      </rPr>
+      <t>as</t>
     </r>
     <r>
       <rPr>
@@ -208,43 +182,21 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t>LastName</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
+      <t xml:space="preserve"> userStartEvent</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>,</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>''</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
         <color theme="1"/>
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> </t>
+      <t xml:space="preserve">[UserEndEvent] </t>
     </r>
     <r>
       <rPr>
@@ -262,31 +214,13 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> lastName</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
+      <t xml:space="preserve"> userEndEvent</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>,</t>
     </r>
-  </si>
-  <si>
-    <r>
-      <t>coalesce</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
     <r>
       <rPr>
         <sz val="10"/>
@@ -294,16 +228,16 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t>h</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
+      <t xml:space="preserve">[RsvpState] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Consolas"/>
+        <family val="2"/>
+      </rPr>
+      <t>as</t>
     </r>
     <r>
       <rPr>
@@ -312,43 +246,21 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t>DisplayName</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
+      <t xml:space="preserve"> rsvpState</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>,</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>''</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
         <color theme="1"/>
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> </t>
+      <t xml:space="preserve">[AttendenceState] </t>
     </r>
     <r>
       <rPr>
@@ -366,31 +278,13 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> dispName</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
+      <t xml:space="preserve"> attendenceState</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>,</t>
     </r>
-  </si>
-  <si>
-    <r>
-      <t>coalesce</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
     <r>
       <rPr>
         <sz val="10"/>
@@ -398,16 +292,16 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t>h</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
+      <t xml:space="preserve">[IsHare] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Consolas"/>
+        <family val="2"/>
+      </rPr>
+      <t>as</t>
     </r>
     <r>
       <rPr>
@@ -416,43 +310,21 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t>HashName</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
+      <t xml:space="preserve"> isHare</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>,</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>''</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
         <color theme="1"/>
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> </t>
+      <t xml:space="preserve">[EventCountOverride] </t>
     </r>
     <r>
       <rPr>
@@ -470,285 +342,18 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> hashName</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>,</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>coalesce</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>h</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>Photo</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>''</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>as</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> photo</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>,</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>coalesce</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>h</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>NameDisplayPreference</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>as</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> dispPref</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>,</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>h</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">id </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>as</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> hasherId</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF808080"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>,</t>
-    </r>
-  </si>
-  <si>
-    <t>HashersTableHelper</t>
+      <t xml:space="preserve"> eventCountOverride</t>
+    </r>
+  </si>
+  <si>
+    <t>HasherEventMapTableHelper</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -782,18 +387,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFF00FF"/>
-      <name val="Consolas"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Consolas"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -821,7 +414,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1170,435 +763,439 @@
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" t="str">
         <f>SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A2," ",REPT(" ",100)),100)),",","")</f>
-        <v>hasherId</v>
+        <v>hemId</v>
       </c>
       <c r="D2" t="str">
         <f>"this."&amp;C2 &amp; ","</f>
-        <v>this.hasherId,</v>
+        <v>this.hemId,</v>
       </c>
       <c r="E2" t="str">
         <f>"final " &amp; VLOOKUP(B2,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C2 &amp; ";"</f>
-        <v>final String hasherId;</v>
+        <v>final String hemId;</v>
       </c>
       <c r="F2" t="str">
         <f t="shared" ref="F2:F21" si="0">C2&amp;": jsonItem['"&amp;C2&amp;"'],"</f>
-        <v>hasherId: jsonItem['hasherId'],</v>
+        <v>hemId: jsonItem['hemId'],</v>
       </c>
       <c r="G2" t="str">
         <f t="shared" ref="G2:G21" si="1">UPPER(MID(C2,1,1)) &amp; MID(C2,2,9999)</f>
-        <v>HasherId</v>
+        <v>HemId</v>
       </c>
       <c r="H2" t="str">
         <f>"col"&amp;G2</f>
-        <v>colHasherId</v>
+        <v>colHemId</v>
       </c>
       <c r="I2" t="str">
         <f t="shared" ref="I2:I21" si="2">"static const String "&amp;H2&amp;"= '"&amp;C2&amp;"';"</f>
-        <v>static const String colHasherId= 'hasherId';</v>
+        <v>static const String colHemId= 'hemId';</v>
       </c>
       <c r="J2" t="str">
         <f t="shared" ref="J2:J21" si="3">"$"&amp;H2&amp;" "&amp;B2&amp;","</f>
-        <v>$colHasherId TEXT NOT NULL,</v>
+        <v>$colHemId TEXT NOT NULL,</v>
       </c>
       <c r="K2" t="str">
         <f t="shared" ref="K2:K21" si="4">$K$1&amp;"."&amp;H2&amp;": item."&amp;C2&amp;","</f>
-        <v>HashersTableHelper.colHasherId: item.hasherId,</v>
+        <v>HasherEventMapTableHelper.colHemId: item.hemId,</v>
       </c>
       <c r="L2" t="str">
         <f t="shared" ref="L2:L21" si="5">C2&amp;": map["&amp;$K$1&amp;"."&amp;H2&amp;"],"</f>
-        <v>hasherId: map[HashersTableHelper.colHasherId],</v>
+        <v>hemId: map[HasherEventMapTableHelper.colHemId],</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3" t="str">
         <f t="shared" ref="C3:C22" si="6">SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A3," ",REPT(" ",100)),100)),",","")</f>
-        <v>firstName</v>
+        <v>userId</v>
       </c>
       <c r="D3" t="str">
         <f t="shared" ref="D3:D22" si="7">"this."&amp;C3 &amp; ","</f>
-        <v>this.firstName,</v>
+        <v>this.userId,</v>
       </c>
       <c r="E3" t="str">
         <f>"final " &amp; VLOOKUP(B3,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C3 &amp; ";"</f>
-        <v>final String firstName;</v>
+        <v>final String userId;</v>
       </c>
       <c r="F3" t="str">
         <f t="shared" si="0"/>
-        <v>firstName: jsonItem['firstName'],</v>
+        <v>userId: jsonItem['userId'],</v>
       </c>
       <c r="G3" t="str">
         <f t="shared" si="1"/>
-        <v>FirstName</v>
+        <v>UserId</v>
       </c>
       <c r="H3" t="str">
         <f t="shared" ref="H3:H21" si="8">"col"&amp;G3</f>
-        <v>colFirstName</v>
+        <v>colUserId</v>
       </c>
       <c r="I3" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colFirstName= 'firstName';</v>
+        <v>static const String colUserId= 'userId';</v>
       </c>
       <c r="J3" t="str">
         <f t="shared" si="3"/>
-        <v>$colFirstName TEXT,</v>
+        <v>$colUserId TEXT NOT NULL,</v>
       </c>
       <c r="K3" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.colFirstName: item.firstName,</v>
+        <v>HasherEventMapTableHelper.colUserId: item.userId,</v>
       </c>
       <c r="L3" t="str">
         <f t="shared" si="5"/>
-        <v>firstName: map[HashersTableHelper.colFirstName],</v>
+        <v>userId: map[HasherEventMapTableHelper.colUserId],</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" t="str">
         <f t="shared" si="6"/>
-        <v>lastName</v>
+        <v>eventId</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" si="7"/>
-        <v>this.lastName,</v>
+        <v>this.eventId,</v>
       </c>
       <c r="E4" t="str">
         <f>"final " &amp; VLOOKUP(B4,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C4 &amp; ";"</f>
-        <v>final String lastName;</v>
+        <v>final String eventId;</v>
       </c>
       <c r="F4" t="str">
         <f t="shared" si="0"/>
-        <v>lastName: jsonItem['lastName'],</v>
+        <v>eventId: jsonItem['eventId'],</v>
       </c>
       <c r="G4" t="str">
         <f t="shared" si="1"/>
-        <v>LastName</v>
+        <v>EventId</v>
       </c>
       <c r="H4" t="str">
         <f t="shared" si="8"/>
-        <v>colLastName</v>
+        <v>colEventId</v>
       </c>
       <c r="I4" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colLastName= 'lastName';</v>
+        <v>static const String colEventId= 'eventId';</v>
       </c>
       <c r="J4" t="str">
         <f t="shared" si="3"/>
-        <v>$colLastName TEXT,</v>
+        <v>$colEventId TEXT NOT NULL,</v>
       </c>
       <c r="K4" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.colLastName: item.lastName,</v>
+        <v>HasherEventMapTableHelper.colEventId: item.eventId,</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="5"/>
-        <v>lastName: map[HashersTableHelper.colLastName],</v>
+        <v>eventId: map[HasherEventMapTableHelper.colEventId],</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="6"/>
-        <v>dispName</v>
+        <v>userStartEvent</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="7"/>
-        <v>this.dispName,</v>
+        <v>this.userStartEvent,</v>
       </c>
       <c r="E5" t="str">
         <f>"final " &amp; VLOOKUP(B5,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C5 &amp; ";"</f>
-        <v>final String dispName;</v>
+        <v>final String userStartEvent;</v>
       </c>
       <c r="F5" t="str">
         <f t="shared" si="0"/>
-        <v>dispName: jsonItem['dispName'],</v>
+        <v>userStartEvent: jsonItem['userStartEvent'],</v>
       </c>
       <c r="G5" t="str">
         <f t="shared" si="1"/>
-        <v>DispName</v>
+        <v>UserStartEvent</v>
       </c>
       <c r="H5" t="str">
         <f t="shared" si="8"/>
-        <v>colDispName</v>
+        <v>colUserStartEvent</v>
       </c>
       <c r="I5" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colDispName= 'dispName';</v>
+        <v>static const String colUserStartEvent= 'userStartEvent';</v>
       </c>
       <c r="J5" t="str">
         <f t="shared" si="3"/>
-        <v>$colDispName TEXT,</v>
+        <v>$colUserStartEvent TEXT,</v>
       </c>
       <c r="K5" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.colDispName: item.dispName,</v>
+        <v>HasherEventMapTableHelper.colUserStartEvent: item.userStartEvent,</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="5"/>
-        <v>dispName: map[HashersTableHelper.colDispName],</v>
+        <v>userStartEvent: map[HasherEventMapTableHelper.colUserStartEvent],</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="6"/>
-        <v>hashName</v>
+        <v>userEndEvent</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="7"/>
-        <v>this.hashName,</v>
+        <v>this.userEndEvent,</v>
       </c>
       <c r="E6" t="str">
         <f>"final " &amp; VLOOKUP(B6,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C6 &amp; ";"</f>
-        <v>final String hashName;</v>
+        <v>final String userEndEvent;</v>
       </c>
       <c r="F6" t="str">
         <f t="shared" si="0"/>
-        <v>hashName: jsonItem['hashName'],</v>
+        <v>userEndEvent: jsonItem['userEndEvent'],</v>
       </c>
       <c r="G6" t="str">
         <f t="shared" si="1"/>
-        <v>HashName</v>
+        <v>UserEndEvent</v>
       </c>
       <c r="H6" t="str">
         <f t="shared" si="8"/>
-        <v>colHashName</v>
+        <v>colUserEndEvent</v>
       </c>
       <c r="I6" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colHashName= 'hashName';</v>
+        <v>static const String colUserEndEvent= 'userEndEvent';</v>
       </c>
       <c r="J6" t="str">
         <f t="shared" si="3"/>
-        <v>$colHashName TEXT,</v>
+        <v>$colUserEndEvent TEXT,</v>
       </c>
       <c r="K6" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.colHashName: item.hashName,</v>
+        <v>HasherEventMapTableHelper.colUserEndEvent: item.userEndEvent,</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="5"/>
-        <v>hashName: map[HashersTableHelper.colHashName],</v>
+        <v>userEndEvent: map[HasherEventMapTableHelper.colUserEndEvent],</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="6"/>
-        <v>photo</v>
+        <v>rsvpState</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="7"/>
-        <v>this.photo,</v>
+        <v>this.rsvpState,</v>
       </c>
       <c r="E7" t="str">
         <f>"final " &amp; VLOOKUP(B7,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C7 &amp; ";"</f>
-        <v>final String photo;</v>
+        <v>final int rsvpState;</v>
       </c>
       <c r="F7" t="str">
         <f t="shared" si="0"/>
-        <v>photo: jsonItem['photo'],</v>
+        <v>rsvpState: jsonItem['rsvpState'],</v>
       </c>
       <c r="G7" t="str">
         <f t="shared" si="1"/>
-        <v>Photo</v>
+        <v>RsvpState</v>
       </c>
       <c r="H7" t="str">
         <f t="shared" si="8"/>
-        <v>colPhoto</v>
+        <v>colRsvpState</v>
       </c>
       <c r="I7" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colPhoto= 'photo';</v>
+        <v>static const String colRsvpState= 'rsvpState';</v>
       </c>
       <c r="J7" t="str">
         <f t="shared" si="3"/>
-        <v>$colPhoto TEXT,</v>
+        <v>$colRsvpState INT,</v>
       </c>
       <c r="K7" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.colPhoto: item.photo,</v>
+        <v>HasherEventMapTableHelper.colRsvpState: item.rsvpState,</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="5"/>
-        <v>photo: map[HashersTableHelper.colPhoto],</v>
+        <v>rsvpState: map[HasherEventMapTableHelper.colRsvpState],</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="6"/>
-        <v>dispPref</v>
+        <v>attendenceState</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="7"/>
-        <v>this.dispPref,</v>
+        <v>this.attendenceState,</v>
       </c>
       <c r="E8" t="str">
         <f>"final " &amp; VLOOKUP(B8,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C8 &amp; ";"</f>
-        <v>final int dispPref;</v>
+        <v>final int attendenceState;</v>
       </c>
       <c r="F8" t="str">
         <f t="shared" si="0"/>
-        <v>dispPref: jsonItem['dispPref'],</v>
+        <v>attendenceState: jsonItem['attendenceState'],</v>
       </c>
       <c r="G8" t="str">
         <f t="shared" si="1"/>
-        <v>DispPref</v>
+        <v>AttendenceState</v>
       </c>
       <c r="H8" t="str">
         <f t="shared" si="8"/>
-        <v>colDispPref</v>
+        <v>colAttendenceState</v>
       </c>
       <c r="I8" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colDispPref= 'dispPref';</v>
+        <v>static const String colAttendenceState= 'attendenceState';</v>
       </c>
       <c r="J8" t="str">
         <f t="shared" si="3"/>
-        <v>$colDispPref INT,</v>
+        <v>$colAttendenceState INT,</v>
       </c>
       <c r="K8" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.colDispPref: item.dispPref,</v>
+        <v>HasherEventMapTableHelper.colAttendenceState: item.attendenceState,</v>
       </c>
       <c r="L8" t="str">
         <f t="shared" si="5"/>
-        <v>dispPref: map[HashersTableHelper.colDispPref],</v>
+        <v>attendenceState: map[HasherEventMapTableHelper.colAttendenceState],</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="1"/>
+      <c r="A9" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="6"/>
-        <v/>
+        <v>isHare</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="7"/>
-        <v>this.,</v>
+        <v>this.isHare,</v>
       </c>
       <c r="E9" t="str">
         <f>"final " &amp; VLOOKUP(B9,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C9 &amp; ";"</f>
-        <v>final int ;</v>
+        <v>final int isHare;</v>
       </c>
       <c r="F9" t="str">
         <f t="shared" si="0"/>
-        <v>: jsonItem[''],</v>
+        <v>isHare: jsonItem['isHare'],</v>
       </c>
       <c r="G9" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>IsHare</v>
       </c>
       <c r="H9" t="str">
         <f t="shared" si="8"/>
-        <v>col</v>
+        <v>colIsHare</v>
       </c>
       <c r="I9" t="str">
         <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <v>static const String colIsHare= 'isHare';</v>
       </c>
       <c r="J9" t="str">
         <f t="shared" si="3"/>
-        <v>$col INT,</v>
+        <v>$colIsHare INT,</v>
       </c>
       <c r="K9" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.colIsHare: item.isHare,</v>
       </c>
       <c r="L9" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>isHare: map[HasherEventMapTableHelper.colIsHare],</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="1"/>
+      <c r="A10" s="3" t="s">
+        <v>21</v>
+      </c>
       <c r="B10" t="s">
         <v>5</v>
       </c>
       <c r="C10" t="str">
         <f t="shared" si="6"/>
-        <v/>
+        <v>eventCountOverride</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="7"/>
-        <v>this.,</v>
+        <v>this.eventCountOverride,</v>
       </c>
       <c r="E10" t="str">
         <f>"final " &amp; VLOOKUP(B10,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C10 &amp; ";"</f>
-        <v>final num ;</v>
+        <v>final num eventCountOverride;</v>
       </c>
       <c r="F10" t="str">
         <f t="shared" si="0"/>
-        <v>: jsonItem[''],</v>
+        <v>eventCountOverride: jsonItem['eventCountOverride'],</v>
       </c>
       <c r="G10" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>EventCountOverride</v>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="8"/>
-        <v>col</v>
+        <v>colEventCountOverride</v>
       </c>
       <c r="I10" t="str">
         <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <v>static const String colEventCountOverride= 'eventCountOverride';</v>
       </c>
       <c r="J10" t="str">
         <f t="shared" si="3"/>
-        <v>$col NUM,</v>
+        <v>$colEventCountOverride NUM,</v>
       </c>
       <c r="K10" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.colEventCountOverride: item.eventCountOverride,</v>
       </c>
       <c r="L10" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>eventCountOverride: map[HasherEventMapTableHelper.colEventCountOverride],</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -1640,11 +1237,11 @@
       </c>
       <c r="K11" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.col: item.,</v>
       </c>
       <c r="L11" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>: map[HasherEventMapTableHelper.col],</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
@@ -1686,11 +1283,11 @@
       </c>
       <c r="K12" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.col: item.,</v>
       </c>
       <c r="L12" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>: map[HasherEventMapTableHelper.col],</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
@@ -1732,11 +1329,11 @@
       </c>
       <c r="K13" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.col: item.,</v>
       </c>
       <c r="L13" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>: map[HasherEventMapTableHelper.col],</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
@@ -1773,11 +1370,11 @@
       </c>
       <c r="K14" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.col: item.,</v>
       </c>
       <c r="L14" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>: map[HasherEventMapTableHelper.col],</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
@@ -1814,11 +1411,11 @@
       </c>
       <c r="K15" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.col: item.,</v>
       </c>
       <c r="L15" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>: map[HasherEventMapTableHelper.col],</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
@@ -1855,11 +1452,11 @@
       </c>
       <c r="K16" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.col: item.,</v>
       </c>
       <c r="L16" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>: map[HasherEventMapTableHelper.col],</v>
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.2">
@@ -1896,11 +1493,11 @@
       </c>
       <c r="K17" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.col: item.,</v>
       </c>
       <c r="L17" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>: map[HasherEventMapTableHelper.col],</v>
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.2">
@@ -1937,11 +1534,11 @@
       </c>
       <c r="K18" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.col: item.,</v>
       </c>
       <c r="L18" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>: map[HasherEventMapTableHelper.col],</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.2">
@@ -1978,11 +1575,11 @@
       </c>
       <c r="K19" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.col: item.,</v>
       </c>
       <c r="L19" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>: map[HasherEventMapTableHelper.col],</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.2">
@@ -2019,11 +1616,11 @@
       </c>
       <c r="K20" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.col: item.,</v>
       </c>
       <c r="L20" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>: map[HasherEventMapTableHelper.col],</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.2">
@@ -2060,11 +1657,11 @@
       </c>
       <c r="K21" t="str">
         <f t="shared" si="4"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <v>HasherEventMapTableHelper.col: item.,</v>
       </c>
       <c r="L21" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <v>: map[HasherEventMapTableHelper.col],</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Intermediate: Extended receipts data model to include reimbursements
</commit_message>
<xml_diff>
--- a/android/devHelpers/DataClassHelper.xlsx
+++ b/android/devHelpers/DataClassHelper.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jameswhite/Projects/flutter/HC/HarrierCentral/HarrierCentralMobile-Flutter/android/devHelpers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E195015F-4387-644F-853A-B2CCED30F208}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61956AE7-E3F8-764F-AB32-D3AE708D1261}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="20540" xr2:uid="{50A37692-8663-7F4C-91F6-2AE3BA380A00}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="20">
   <si>
     <t>wireName</t>
   </si>
@@ -68,7 +68,16 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">[id] </t>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Consolas"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">[Notes] </t>
     </r>
     <r>
       <rPr>
@@ -86,7 +95,7 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> hemId</t>
+      <t xml:space="preserve"> notes</t>
     </r>
   </si>
   <si>
@@ -100,7 +109,7 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">[UserId] </t>
+      <t xml:space="preserve">[ReimbursedBy] </t>
     </r>
     <r>
       <rPr>
@@ -118,7 +127,7 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> userId</t>
+      <t xml:space="preserve"> reimbursedBy</t>
     </r>
   </si>
   <si>
@@ -132,7 +141,7 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">[EventId] </t>
+      <t xml:space="preserve">[ReimbursedOn] </t>
     </r>
     <r>
       <rPr>
@@ -150,7 +159,7 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> eventId</t>
+      <t xml:space="preserve"> reimbursedOn</t>
     </r>
   </si>
   <si>
@@ -164,7 +173,7 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">[UserStartEvent] </t>
+      <t xml:space="preserve">[ReimbursedAmount] </t>
     </r>
     <r>
       <rPr>
@@ -182,7 +191,7 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> userStartEvent</t>
+      <t xml:space="preserve"> reimbursedAmount</t>
     </r>
   </si>
   <si>
@@ -196,7 +205,7 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">[UserEndEvent] </t>
+      <t xml:space="preserve">[ReimbursedNotes] </t>
     </r>
     <r>
       <rPr>
@@ -214,139 +223,14 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> userEndEvent</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">[RsvpState] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>as</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> rsvpState</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">[AttendenceState] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>as</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> attendenceState</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">[IsHare] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>as</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> isHare</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">[EventCountOverride] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>as</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> eventCountOverride</t>
-    </r>
-  </si>
-  <si>
-    <t>HasherEventMapTableHelper</t>
+      <t xml:space="preserve"> reimbursedNotes</t>
+    </r>
+  </si>
+  <si>
+    <t>ReceiptsTableHelper</t>
+  </si>
+  <si>
+    <t>{ name: 'receiptAmount', value: req.body.receiptAmount },</t>
   </si>
 </sst>
 </file>
@@ -729,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447EABA0-45A3-CE41-BCC1-A3347CEBD28F}">
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="55.33203125" customWidth="1"/>
@@ -741,9 +625,10 @@
     <col min="9" max="9" width="71" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="34.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="75.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="61" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
@@ -763,202 +648,221 @@
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" t="str">
         <f>SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A2," ",REPT(" ",100)),100)),",","")</f>
-        <v>hemId</v>
+        <v>notes</v>
       </c>
       <c r="D2" t="str">
         <f>"this."&amp;C2 &amp; ","</f>
-        <v>this.hemId,</v>
+        <v>this.notes,</v>
       </c>
       <c r="E2" t="str">
         <f>"final " &amp; VLOOKUP(B2,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C2 &amp; ";"</f>
-        <v>final String hemId;</v>
+        <v>final String notes;</v>
       </c>
       <c r="F2" t="str">
         <f t="shared" ref="F2:F21" si="0">C2&amp;": jsonItem['"&amp;C2&amp;"'],"</f>
-        <v>hemId: jsonItem['hemId'],</v>
+        <v>notes: jsonItem['notes'],</v>
       </c>
       <c r="G2" t="str">
         <f t="shared" ref="G2:G21" si="1">UPPER(MID(C2,1,1)) &amp; MID(C2,2,9999)</f>
-        <v>HemId</v>
+        <v>Notes</v>
       </c>
       <c r="H2" t="str">
         <f>"col"&amp;G2</f>
-        <v>colHemId</v>
+        <v>colNotes</v>
       </c>
       <c r="I2" t="str">
         <f t="shared" ref="I2:I21" si="2">"static const String "&amp;H2&amp;"= '"&amp;C2&amp;"';"</f>
-        <v>static const String colHemId= 'hemId';</v>
+        <v>static const String colNotes= 'notes';</v>
       </c>
       <c r="J2" t="str">
         <f t="shared" ref="J2:J21" si="3">"$"&amp;H2&amp;" "&amp;B2&amp;","</f>
-        <v>$colHemId TEXT NOT NULL,</v>
+        <v>$colNotes TEXT,</v>
       </c>
       <c r="K2" t="str">
         <f t="shared" ref="K2:K21" si="4">$K$1&amp;"."&amp;H2&amp;": item."&amp;C2&amp;","</f>
-        <v>HasherEventMapTableHelper.colHemId: item.hemId,</v>
+        <v>ReceiptsTableHelper.colNotes: item.notes,</v>
       </c>
       <c r="L2" t="str">
         <f t="shared" ref="L2:L21" si="5">C2&amp;": map["&amp;$K$1&amp;"."&amp;H2&amp;"],"</f>
-        <v>hemId: map[HasherEventMapTableHelper.colHemId],</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+        <v>notes: map[ReceiptsTableHelper.colNotes],</v>
+      </c>
+      <c r="M2" t="str">
+        <f>"{ name: '"&amp;C2&amp;"', value: req.body."&amp;C2&amp;" },"</f>
+        <v>{ name: 'notes', value: req.body.notes },</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" t="str">
         <f t="shared" ref="C3:C22" si="6">SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A3," ",REPT(" ",100)),100)),",","")</f>
-        <v>userId</v>
+        <v>reimbursedBy</v>
       </c>
       <c r="D3" t="str">
         <f t="shared" ref="D3:D22" si="7">"this."&amp;C3 &amp; ","</f>
-        <v>this.userId,</v>
+        <v>this.reimbursedBy,</v>
       </c>
       <c r="E3" t="str">
         <f>"final " &amp; VLOOKUP(B3,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C3 &amp; ";"</f>
-        <v>final String userId;</v>
+        <v>final String reimbursedBy;</v>
       </c>
       <c r="F3" t="str">
         <f t="shared" si="0"/>
-        <v>userId: jsonItem['userId'],</v>
+        <v>reimbursedBy: jsonItem['reimbursedBy'],</v>
       </c>
       <c r="G3" t="str">
         <f t="shared" si="1"/>
-        <v>UserId</v>
+        <v>ReimbursedBy</v>
       </c>
       <c r="H3" t="str">
         <f t="shared" ref="H3:H21" si="8">"col"&amp;G3</f>
-        <v>colUserId</v>
+        <v>colReimbursedBy</v>
       </c>
       <c r="I3" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colUserId= 'userId';</v>
+        <v>static const String colReimbursedBy= 'reimbursedBy';</v>
       </c>
       <c r="J3" t="str">
         <f t="shared" si="3"/>
-        <v>$colUserId TEXT NOT NULL,</v>
+        <v>$colReimbursedBy TEXT,</v>
       </c>
       <c r="K3" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.colUserId: item.userId,</v>
+        <v>ReceiptsTableHelper.colReimbursedBy: item.reimbursedBy,</v>
       </c>
       <c r="L3" t="str">
         <f t="shared" si="5"/>
-        <v>userId: map[HasherEventMapTableHelper.colUserId],</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+        <v>reimbursedBy: map[ReceiptsTableHelper.colReimbursedBy],</v>
+      </c>
+      <c r="M3" t="str">
+        <f t="shared" ref="M3:M21" si="9">"{ name: '"&amp;C3&amp;"', value: req.body."&amp;C3&amp;" },"</f>
+        <v>{ name: 'reimbursedBy', value: req.body.reimbursedBy },</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" t="str">
         <f t="shared" si="6"/>
-        <v>eventId</v>
+        <v>reimbursedOn</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" si="7"/>
-        <v>this.eventId,</v>
+        <v>this.reimbursedOn,</v>
       </c>
       <c r="E4" t="str">
         <f>"final " &amp; VLOOKUP(B4,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C4 &amp; ";"</f>
-        <v>final String eventId;</v>
+        <v>final String reimbursedOn;</v>
       </c>
       <c r="F4" t="str">
         <f t="shared" si="0"/>
-        <v>eventId: jsonItem['eventId'],</v>
+        <v>reimbursedOn: jsonItem['reimbursedOn'],</v>
       </c>
       <c r="G4" t="str">
         <f t="shared" si="1"/>
-        <v>EventId</v>
+        <v>ReimbursedOn</v>
       </c>
       <c r="H4" t="str">
         <f t="shared" si="8"/>
-        <v>colEventId</v>
+        <v>colReimbursedOn</v>
       </c>
       <c r="I4" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colEventId= 'eventId';</v>
+        <v>static const String colReimbursedOn= 'reimbursedOn';</v>
       </c>
       <c r="J4" t="str">
         <f t="shared" si="3"/>
-        <v>$colEventId TEXT NOT NULL,</v>
+        <v>$colReimbursedOn TEXT,</v>
       </c>
       <c r="K4" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.colEventId: item.eventId,</v>
+        <v>ReceiptsTableHelper.colReimbursedOn: item.reimbursedOn,</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="5"/>
-        <v>eventId: map[HasherEventMapTableHelper.colEventId],</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+        <v>reimbursedOn: map[ReceiptsTableHelper.colReimbursedOn],</v>
+      </c>
+      <c r="M4" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: 'reimbursedOn', value: req.body.reimbursedOn },</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="6"/>
-        <v>userStartEvent</v>
+        <v>reimbursedAmount</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="7"/>
-        <v>this.userStartEvent,</v>
+        <v>this.reimbursedAmount,</v>
       </c>
       <c r="E5" t="str">
         <f>"final " &amp; VLOOKUP(B5,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C5 &amp; ";"</f>
-        <v>final String userStartEvent;</v>
+        <v>final num reimbursedAmount;</v>
       </c>
       <c r="F5" t="str">
         <f t="shared" si="0"/>
-        <v>userStartEvent: jsonItem['userStartEvent'],</v>
+        <v>reimbursedAmount: jsonItem['reimbursedAmount'],</v>
       </c>
       <c r="G5" t="str">
         <f t="shared" si="1"/>
-        <v>UserStartEvent</v>
+        <v>ReimbursedAmount</v>
       </c>
       <c r="H5" t="str">
         <f t="shared" si="8"/>
-        <v>colUserStartEvent</v>
+        <v>colReimbursedAmount</v>
       </c>
       <c r="I5" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colUserStartEvent= 'userStartEvent';</v>
+        <v>static const String colReimbursedAmount= 'reimbursedAmount';</v>
       </c>
       <c r="J5" t="str">
         <f t="shared" si="3"/>
-        <v>$colUserStartEvent TEXT,</v>
+        <v>$colReimbursedAmount NUM,</v>
       </c>
       <c r="K5" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.colUserStartEvent: item.userStartEvent,</v>
+        <v>ReceiptsTableHelper.colReimbursedAmount: item.reimbursedAmount,</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="5"/>
-        <v>userStartEvent: map[HasherEventMapTableHelper.colUserStartEvent],</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+        <v>reimbursedAmount: map[ReceiptsTableHelper.colReimbursedAmount],</v>
+      </c>
+      <c r="M5" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: 'reimbursedAmount', value: req.body.reimbursedAmount },</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>17</v>
       </c>
@@ -967,238 +871,250 @@
       </c>
       <c r="C6" t="str">
         <f t="shared" si="6"/>
-        <v>userEndEvent</v>
+        <v>reimbursedNotes</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="7"/>
-        <v>this.userEndEvent,</v>
+        <v>this.reimbursedNotes,</v>
       </c>
       <c r="E6" t="str">
         <f>"final " &amp; VLOOKUP(B6,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C6 &amp; ";"</f>
-        <v>final String userEndEvent;</v>
+        <v>final String reimbursedNotes;</v>
       </c>
       <c r="F6" t="str">
         <f t="shared" si="0"/>
-        <v>userEndEvent: jsonItem['userEndEvent'],</v>
+        <v>reimbursedNotes: jsonItem['reimbursedNotes'],</v>
       </c>
       <c r="G6" t="str">
         <f t="shared" si="1"/>
-        <v>UserEndEvent</v>
+        <v>ReimbursedNotes</v>
       </c>
       <c r="H6" t="str">
         <f t="shared" si="8"/>
-        <v>colUserEndEvent</v>
+        <v>colReimbursedNotes</v>
       </c>
       <c r="I6" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colUserEndEvent= 'userEndEvent';</v>
+        <v>static const String colReimbursedNotes= 'reimbursedNotes';</v>
       </c>
       <c r="J6" t="str">
         <f t="shared" si="3"/>
-        <v>$colUserEndEvent TEXT,</v>
+        <v>$colReimbursedNotes TEXT,</v>
       </c>
       <c r="K6" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.colUserEndEvent: item.userEndEvent,</v>
+        <v>ReceiptsTableHelper.colReimbursedNotes: item.reimbursedNotes,</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="5"/>
-        <v>userEndEvent: map[HasherEventMapTableHelper.colUserEndEvent],</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>reimbursedNotes: map[ReceiptsTableHelper.colReimbursedNotes],</v>
+      </c>
+      <c r="M6" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: 'reimbursedNotes', value: req.body.reimbursedNotes },</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A7" s="3"/>
       <c r="B7" t="s">
         <v>4</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="6"/>
-        <v>rsvpState</v>
+        <v/>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="7"/>
-        <v>this.rsvpState,</v>
+        <v>this.,</v>
       </c>
       <c r="E7" t="str">
         <f>"final " &amp; VLOOKUP(B7,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C7 &amp; ";"</f>
-        <v>final int rsvpState;</v>
+        <v>final int ;</v>
       </c>
       <c r="F7" t="str">
         <f t="shared" si="0"/>
-        <v>rsvpState: jsonItem['rsvpState'],</v>
+        <v>: jsonItem[''],</v>
       </c>
       <c r="G7" t="str">
         <f t="shared" si="1"/>
-        <v>RsvpState</v>
+        <v/>
       </c>
       <c r="H7" t="str">
         <f t="shared" si="8"/>
-        <v>colRsvpState</v>
+        <v>col</v>
       </c>
       <c r="I7" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colRsvpState= 'rsvpState';</v>
+        <v>static const String col= '';</v>
       </c>
       <c r="J7" t="str">
         <f t="shared" si="3"/>
-        <v>$colRsvpState INT,</v>
+        <v>$col INT,</v>
       </c>
       <c r="K7" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.colRsvpState: item.rsvpState,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="5"/>
-        <v>rsvpState: map[HasherEventMapTableHelper.colRsvpState],</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>19</v>
-      </c>
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M7" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" s="3"/>
       <c r="B8" t="s">
         <v>4</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="6"/>
-        <v>attendenceState</v>
+        <v/>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="7"/>
-        <v>this.attendenceState,</v>
+        <v>this.,</v>
       </c>
       <c r="E8" t="str">
         <f>"final " &amp; VLOOKUP(B8,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C8 &amp; ";"</f>
-        <v>final int attendenceState;</v>
+        <v>final int ;</v>
       </c>
       <c r="F8" t="str">
         <f t="shared" si="0"/>
-        <v>attendenceState: jsonItem['attendenceState'],</v>
+        <v>: jsonItem[''],</v>
       </c>
       <c r="G8" t="str">
         <f t="shared" si="1"/>
-        <v>AttendenceState</v>
+        <v/>
       </c>
       <c r="H8" t="str">
         <f t="shared" si="8"/>
-        <v>colAttendenceState</v>
+        <v>col</v>
       </c>
       <c r="I8" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colAttendenceState= 'attendenceState';</v>
+        <v>static const String col= '';</v>
       </c>
       <c r="J8" t="str">
         <f t="shared" si="3"/>
-        <v>$colAttendenceState INT,</v>
+        <v>$col INT,</v>
       </c>
       <c r="K8" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.colAttendenceState: item.attendenceState,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L8" t="str">
         <f t="shared" si="5"/>
-        <v>attendenceState: map[HasherEventMapTableHelper.colAttendenceState],</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>20</v>
-      </c>
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M8" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" s="3"/>
       <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="6"/>
-        <v>isHare</v>
+        <v/>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="7"/>
-        <v>this.isHare,</v>
+        <v>this.,</v>
       </c>
       <c r="E9" t="str">
         <f>"final " &amp; VLOOKUP(B9,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C9 &amp; ";"</f>
-        <v>final int isHare;</v>
+        <v>final int ;</v>
       </c>
       <c r="F9" t="str">
         <f t="shared" si="0"/>
-        <v>isHare: jsonItem['isHare'],</v>
+        <v>: jsonItem[''],</v>
       </c>
       <c r="G9" t="str">
         <f t="shared" si="1"/>
-        <v>IsHare</v>
+        <v/>
       </c>
       <c r="H9" t="str">
         <f t="shared" si="8"/>
-        <v>colIsHare</v>
+        <v>col</v>
       </c>
       <c r="I9" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colIsHare= 'isHare';</v>
+        <v>static const String col= '';</v>
       </c>
       <c r="J9" t="str">
         <f t="shared" si="3"/>
-        <v>$colIsHare INT,</v>
+        <v>$col INT,</v>
       </c>
       <c r="K9" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.colIsHare: item.isHare,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L9" t="str">
         <f t="shared" si="5"/>
-        <v>isHare: map[HasherEventMapTableHelper.colIsHare],</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>21</v>
-      </c>
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M9" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" s="3"/>
       <c r="B10" t="s">
         <v>5</v>
       </c>
       <c r="C10" t="str">
         <f t="shared" si="6"/>
-        <v>eventCountOverride</v>
+        <v/>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="7"/>
-        <v>this.eventCountOverride,</v>
+        <v>this.,</v>
       </c>
       <c r="E10" t="str">
         <f>"final " &amp; VLOOKUP(B10,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C10 &amp; ";"</f>
-        <v>final num eventCountOverride;</v>
+        <v>final num ;</v>
       </c>
       <c r="F10" t="str">
         <f t="shared" si="0"/>
-        <v>eventCountOverride: jsonItem['eventCountOverride'],</v>
+        <v>: jsonItem[''],</v>
       </c>
       <c r="G10" t="str">
         <f t="shared" si="1"/>
-        <v>EventCountOverride</v>
+        <v/>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="8"/>
-        <v>colEventCountOverride</v>
+        <v>col</v>
       </c>
       <c r="I10" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colEventCountOverride= 'eventCountOverride';</v>
+        <v>static const String col= '';</v>
       </c>
       <c r="J10" t="str">
         <f t="shared" si="3"/>
-        <v>$colEventCountOverride NUM,</v>
+        <v>$col NUM,</v>
       </c>
       <c r="K10" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.colEventCountOverride: item.eventCountOverride,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L10" t="str">
         <f t="shared" si="5"/>
-        <v>eventCountOverride: map[HasherEventMapTableHelper.colEventCountOverride],</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M10" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" t="s">
         <v>5</v>
@@ -1237,14 +1153,18 @@
       </c>
       <c r="K11" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.col: item.,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L11" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HasherEventMapTableHelper.col],</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M11" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
       <c r="B12" t="s">
         <v>4</v>
@@ -1283,14 +1203,18 @@
       </c>
       <c r="K12" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.col: item.,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L12" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HasherEventMapTableHelper.col],</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M12" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" t="s">
         <v>3</v>
@@ -1329,14 +1253,18 @@
       </c>
       <c r="K13" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.col: item.,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L13" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HasherEventMapTableHelper.col],</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M13" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>4</v>
       </c>
@@ -1370,14 +1298,18 @@
       </c>
       <c r="K14" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.col: item.,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L14" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HasherEventMapTableHelper.col],</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M14" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>5</v>
       </c>
@@ -1411,14 +1343,18 @@
       </c>
       <c r="K15" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.col: item.,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L15" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HasherEventMapTableHelper.col],</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M15" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
         <v>5</v>
       </c>
@@ -1452,14 +1388,18 @@
       </c>
       <c r="K16" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.col: item.,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L16" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HasherEventMapTableHelper.col],</v>
-      </c>
-    </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M16" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>5</v>
       </c>
@@ -1493,14 +1433,18 @@
       </c>
       <c r="K17" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.col: item.,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L17" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HasherEventMapTableHelper.col],</v>
-      </c>
-    </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M17" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>5</v>
       </c>
@@ -1534,14 +1478,18 @@
       </c>
       <c r="K18" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.col: item.,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L18" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HasherEventMapTableHelper.col],</v>
-      </c>
-    </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M18" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>3</v>
       </c>
@@ -1575,14 +1523,18 @@
       </c>
       <c r="K19" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.col: item.,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L19" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HasherEventMapTableHelper.col],</v>
-      </c>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M19" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>3</v>
       </c>
@@ -1616,14 +1568,18 @@
       </c>
       <c r="K20" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.col: item.,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L20" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HasherEventMapTableHelper.col],</v>
-      </c>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M20" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
         <v>4</v>
       </c>
@@ -1657,14 +1613,18 @@
       </c>
       <c r="K21" t="str">
         <f t="shared" si="4"/>
-        <v>HasherEventMapTableHelper.col: item.,</v>
+        <v>ReceiptsTableHelper.col: item.,</v>
       </c>
       <c r="L21" t="str">
         <f t="shared" si="5"/>
-        <v>: map[HasherEventMapTableHelper.col],</v>
-      </c>
-    </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.2">
+        <v>: map[ReceiptsTableHelper.col],</v>
+      </c>
+      <c r="M21" t="str">
+        <f t="shared" si="9"/>
+        <v>{ name: '', value: req.body. },</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.2">
       <c r="C22" t="str">
         <f t="shared" si="6"/>
         <v/>

</xml_diff>

<commit_message>
Intermediate: More migration to HC3 and SQFLITE
</commit_message>
<xml_diff>
--- a/android/devHelpers/DataClassHelper.xlsx
+++ b/android/devHelpers/DataClassHelper.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jameswhite/Projects/flutter/HC/HarrierCentral/HarrierCentralMobile-Flutter/android/devHelpers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61956AE7-E3F8-764F-AB32-D3AE708D1261}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6B17DC-670F-9A43-ACA6-31B25063200B}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="20540" xr2:uid="{50A37692-8663-7F4C-91F6-2AE3BA380A00}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="17">
   <si>
     <t>wireName</t>
   </si>
@@ -67,6 +67,9 @@
     <t>num</t>
   </si>
   <si>
+    <t>{ name: 'receiptAmount', value: req.body.receiptAmount },</t>
+  </si>
+  <si>
     <r>
       <t>,</t>
     </r>
@@ -77,7 +80,25 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">[Notes] </t>
+      <t>evt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF808080"/>
+        <rFont val="Consolas"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Consolas"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">[EventPriceForMembers] </t>
     </r>
     <r>
       <rPr>
@@ -95,7 +116,7 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> notes</t>
+      <t xml:space="preserve"> eventPriceForMembers</t>
     </r>
   </si>
   <si>
@@ -109,7 +130,25 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">[ReimbursedBy] </t>
+      <t>evt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF808080"/>
+        <rFont val="Consolas"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Consolas"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">[EventPriceForNonMembers] </t>
     </r>
     <r>
       <rPr>
@@ -127,110 +166,11 @@
         <rFont val="Consolas"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> reimbursedBy</t>
+      <t xml:space="preserve"> eventPriceForNonMembers</t>
     </r>
   </si>
   <si>
-    <r>
-      <t>,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">[ReimbursedOn] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>as</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> reimbursedOn</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">[ReimbursedAmount] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>as</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> reimbursedAmount</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">[ReimbursedNotes] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t>as</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Consolas"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> reimbursedNotes</t>
-    </r>
-  </si>
-  <si>
-    <t>ReceiptsTableHelper</t>
-  </si>
-  <si>
-    <t>{ name: 'receiptAmount', value: req.body.receiptAmount },</t>
+    <t>NarrowEventsTableHelper</t>
   </si>
 </sst>
 </file>
@@ -648,270 +588,264 @@
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C2" t="str">
         <f>SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A2," ",REPT(" ",100)),100)),",","")</f>
-        <v>notes</v>
+        <v>eventPriceForMembers</v>
       </c>
       <c r="D2" t="str">
         <f>"this."&amp;C2 &amp; ","</f>
-        <v>this.notes,</v>
+        <v>this.eventPriceForMembers,</v>
       </c>
       <c r="E2" t="str">
         <f>"final " &amp; VLOOKUP(B2,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C2 &amp; ";"</f>
-        <v>final String notes;</v>
+        <v>final num eventPriceForMembers;</v>
       </c>
       <c r="F2" t="str">
         <f t="shared" ref="F2:F21" si="0">C2&amp;": jsonItem['"&amp;C2&amp;"'],"</f>
-        <v>notes: jsonItem['notes'],</v>
+        <v>eventPriceForMembers: jsonItem['eventPriceForMembers'],</v>
       </c>
       <c r="G2" t="str">
         <f t="shared" ref="G2:G21" si="1">UPPER(MID(C2,1,1)) &amp; MID(C2,2,9999)</f>
-        <v>Notes</v>
+        <v>EventPriceForMembers</v>
       </c>
       <c r="H2" t="str">
         <f>"col"&amp;G2</f>
-        <v>colNotes</v>
+        <v>colEventPriceForMembers</v>
       </c>
       <c r="I2" t="str">
         <f t="shared" ref="I2:I21" si="2">"static const String "&amp;H2&amp;"= '"&amp;C2&amp;"';"</f>
-        <v>static const String colNotes= 'notes';</v>
+        <v>static const String colEventPriceForMembers= 'eventPriceForMembers';</v>
       </c>
       <c r="J2" t="str">
         <f t="shared" ref="J2:J21" si="3">"$"&amp;H2&amp;" "&amp;B2&amp;","</f>
-        <v>$colNotes TEXT,</v>
+        <v>$colEventPriceForMembers NUM,</v>
       </c>
       <c r="K2" t="str">
         <f t="shared" ref="K2:K21" si="4">$K$1&amp;"."&amp;H2&amp;": item."&amp;C2&amp;","</f>
-        <v>ReceiptsTableHelper.colNotes: item.notes,</v>
+        <v>NarrowEventsTableHelper.colEventPriceForMembers: item.eventPriceForMembers,</v>
       </c>
       <c r="L2" t="str">
         <f t="shared" ref="L2:L21" si="5">C2&amp;": map["&amp;$K$1&amp;"."&amp;H2&amp;"],"</f>
-        <v>notes: map[ReceiptsTableHelper.colNotes],</v>
+        <v>eventPriceForMembers: map[NarrowEventsTableHelper.colEventPriceForMembers],</v>
       </c>
       <c r="M2" t="str">
         <f>"{ name: '"&amp;C2&amp;"', value: req.body."&amp;C2&amp;" },"</f>
-        <v>{ name: 'notes', value: req.body.notes },</v>
+        <v>{ name: 'eventPriceForMembers', value: req.body.eventPriceForMembers },</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" t="str">
         <f t="shared" ref="C3:C22" si="6">SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A3," ",REPT(" ",100)),100)),",","")</f>
-        <v>reimbursedBy</v>
+        <v>eventPriceForNonMembers</v>
       </c>
       <c r="D3" t="str">
         <f t="shared" ref="D3:D22" si="7">"this."&amp;C3 &amp; ","</f>
-        <v>this.reimbursedBy,</v>
+        <v>this.eventPriceForNonMembers,</v>
       </c>
       <c r="E3" t="str">
         <f>"final " &amp; VLOOKUP(B3,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C3 &amp; ";"</f>
-        <v>final String reimbursedBy;</v>
+        <v>final num eventPriceForNonMembers;</v>
       </c>
       <c r="F3" t="str">
         <f t="shared" si="0"/>
-        <v>reimbursedBy: jsonItem['reimbursedBy'],</v>
+        <v>eventPriceForNonMembers: jsonItem['eventPriceForNonMembers'],</v>
       </c>
       <c r="G3" t="str">
         <f t="shared" si="1"/>
-        <v>ReimbursedBy</v>
+        <v>EventPriceForNonMembers</v>
       </c>
       <c r="H3" t="str">
         <f t="shared" ref="H3:H21" si="8">"col"&amp;G3</f>
-        <v>colReimbursedBy</v>
+        <v>colEventPriceForNonMembers</v>
       </c>
       <c r="I3" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colReimbursedBy= 'reimbursedBy';</v>
+        <v>static const String colEventPriceForNonMembers= 'eventPriceForNonMembers';</v>
       </c>
       <c r="J3" t="str">
         <f t="shared" si="3"/>
-        <v>$colReimbursedBy TEXT,</v>
+        <v>$colEventPriceForNonMembers NUM,</v>
       </c>
       <c r="K3" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.colReimbursedBy: item.reimbursedBy,</v>
+        <v>NarrowEventsTableHelper.colEventPriceForNonMembers: item.eventPriceForNonMembers,</v>
       </c>
       <c r="L3" t="str">
         <f t="shared" si="5"/>
-        <v>reimbursedBy: map[ReceiptsTableHelper.colReimbursedBy],</v>
+        <v>eventPriceForNonMembers: map[NarrowEventsTableHelper.colEventPriceForNonMembers],</v>
       </c>
       <c r="M3" t="str">
         <f t="shared" ref="M3:M21" si="9">"{ name: '"&amp;C3&amp;"', value: req.body."&amp;C3&amp;" },"</f>
-        <v>{ name: 'reimbursedBy', value: req.body.reimbursedBy },</v>
+        <v>{ name: 'eventPriceForNonMembers', value: req.body.eventPriceForNonMembers },</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="A4" s="3"/>
       <c r="B4" t="s">
         <v>3</v>
       </c>
       <c r="C4" t="str">
         <f t="shared" si="6"/>
-        <v>reimbursedOn</v>
+        <v/>
       </c>
       <c r="D4" t="str">
         <f t="shared" si="7"/>
-        <v>this.reimbursedOn,</v>
+        <v>this.,</v>
       </c>
       <c r="E4" t="str">
         <f>"final " &amp; VLOOKUP(B4,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C4 &amp; ";"</f>
-        <v>final String reimbursedOn;</v>
+        <v>final String ;</v>
       </c>
       <c r="F4" t="str">
         <f t="shared" si="0"/>
-        <v>reimbursedOn: jsonItem['reimbursedOn'],</v>
+        <v>: jsonItem[''],</v>
       </c>
       <c r="G4" t="str">
         <f t="shared" si="1"/>
-        <v>ReimbursedOn</v>
+        <v/>
       </c>
       <c r="H4" t="str">
         <f t="shared" si="8"/>
-        <v>colReimbursedOn</v>
+        <v>col</v>
       </c>
       <c r="I4" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colReimbursedOn= 'reimbursedOn';</v>
+        <v>static const String col= '';</v>
       </c>
       <c r="J4" t="str">
         <f t="shared" si="3"/>
-        <v>$colReimbursedOn TEXT,</v>
+        <v>$col TEXT,</v>
       </c>
       <c r="K4" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.colReimbursedOn: item.reimbursedOn,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="5"/>
-        <v>reimbursedOn: map[ReceiptsTableHelper.colReimbursedOn],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M4" t="str">
         <f t="shared" si="9"/>
-        <v>{ name: 'reimbursedOn', value: req.body.reimbursedOn },</v>
+        <v>{ name: '', value: req.body. },</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="A5" s="3"/>
       <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="6"/>
-        <v>reimbursedAmount</v>
+        <v/>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="7"/>
-        <v>this.reimbursedAmount,</v>
+        <v>this.,</v>
       </c>
       <c r="E5" t="str">
         <f>"final " &amp; VLOOKUP(B5,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C5 &amp; ";"</f>
-        <v>final num reimbursedAmount;</v>
+        <v>final num ;</v>
       </c>
       <c r="F5" t="str">
         <f t="shared" si="0"/>
-        <v>reimbursedAmount: jsonItem['reimbursedAmount'],</v>
+        <v>: jsonItem[''],</v>
       </c>
       <c r="G5" t="str">
         <f t="shared" si="1"/>
-        <v>ReimbursedAmount</v>
+        <v/>
       </c>
       <c r="H5" t="str">
         <f t="shared" si="8"/>
-        <v>colReimbursedAmount</v>
+        <v>col</v>
       </c>
       <c r="I5" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colReimbursedAmount= 'reimbursedAmount';</v>
+        <v>static const String col= '';</v>
       </c>
       <c r="J5" t="str">
         <f t="shared" si="3"/>
-        <v>$colReimbursedAmount NUM,</v>
+        <v>$col NUM,</v>
       </c>
       <c r="K5" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.colReimbursedAmount: item.reimbursedAmount,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="5"/>
-        <v>reimbursedAmount: map[ReceiptsTableHelper.colReimbursedAmount],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M5" t="str">
         <f t="shared" si="9"/>
-        <v>{ name: 'reimbursedAmount', value: req.body.reimbursedAmount },</v>
+        <v>{ name: '', value: req.body. },</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>17</v>
-      </c>
+      <c r="A6" s="3"/>
       <c r="B6" t="s">
         <v>3</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="6"/>
-        <v>reimbursedNotes</v>
+        <v/>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="7"/>
-        <v>this.reimbursedNotes,</v>
+        <v>this.,</v>
       </c>
       <c r="E6" t="str">
         <f>"final " &amp; VLOOKUP(B6,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C6 &amp; ";"</f>
-        <v>final String reimbursedNotes;</v>
+        <v>final String ;</v>
       </c>
       <c r="F6" t="str">
         <f t="shared" si="0"/>
-        <v>reimbursedNotes: jsonItem['reimbursedNotes'],</v>
+        <v>: jsonItem[''],</v>
       </c>
       <c r="G6" t="str">
         <f t="shared" si="1"/>
-        <v>ReimbursedNotes</v>
+        <v/>
       </c>
       <c r="H6" t="str">
         <f t="shared" si="8"/>
-        <v>colReimbursedNotes</v>
+        <v>col</v>
       </c>
       <c r="I6" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colReimbursedNotes= 'reimbursedNotes';</v>
+        <v>static const String col= '';</v>
       </c>
       <c r="J6" t="str">
         <f t="shared" si="3"/>
-        <v>$colReimbursedNotes TEXT,</v>
+        <v>$col TEXT,</v>
       </c>
       <c r="K6" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.colReimbursedNotes: item.reimbursedNotes,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="5"/>
-        <v>reimbursedNotes: map[ReceiptsTableHelper.colReimbursedNotes],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M6" t="str">
         <f t="shared" si="9"/>
-        <v>{ name: 'reimbursedNotes', value: req.body.reimbursedNotes },</v>
+        <v>{ name: '', value: req.body. },</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -953,11 +887,11 @@
       </c>
       <c r="K7" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M7" t="str">
         <f t="shared" si="9"/>
@@ -1003,11 +937,11 @@
       </c>
       <c r="K8" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L8" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M8" t="str">
         <f t="shared" si="9"/>
@@ -1053,11 +987,11 @@
       </c>
       <c r="K9" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L9" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M9" t="str">
         <f t="shared" si="9"/>
@@ -1103,11 +1037,11 @@
       </c>
       <c r="K10" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L10" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M10" t="str">
         <f t="shared" si="9"/>
@@ -1153,11 +1087,11 @@
       </c>
       <c r="K11" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L11" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M11" t="str">
         <f t="shared" si="9"/>
@@ -1203,11 +1137,11 @@
       </c>
       <c r="K12" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L12" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M12" t="str">
         <f t="shared" si="9"/>
@@ -1253,11 +1187,11 @@
       </c>
       <c r="K13" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L13" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M13" t="str">
         <f t="shared" si="9"/>
@@ -1298,11 +1232,11 @@
       </c>
       <c r="K14" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L14" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M14" t="str">
         <f t="shared" si="9"/>
@@ -1343,11 +1277,11 @@
       </c>
       <c r="K15" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L15" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M15" t="str">
         <f t="shared" si="9"/>
@@ -1388,11 +1322,11 @@
       </c>
       <c r="K16" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L16" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M16" t="str">
         <f t="shared" si="9"/>
@@ -1433,11 +1367,11 @@
       </c>
       <c r="K17" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L17" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M17" t="str">
         <f t="shared" si="9"/>
@@ -1478,11 +1412,11 @@
       </c>
       <c r="K18" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L18" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M18" t="str">
         <f t="shared" si="9"/>
@@ -1523,11 +1457,11 @@
       </c>
       <c r="K19" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L19" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M19" t="str">
         <f t="shared" si="9"/>
@@ -1568,11 +1502,11 @@
       </c>
       <c r="K20" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L20" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M20" t="str">
         <f t="shared" si="9"/>
@@ -1613,11 +1547,11 @@
       </c>
       <c r="K21" t="str">
         <f t="shared" si="4"/>
-        <v>ReceiptsTableHelper.col: item.,</v>
+        <v>NarrowEventsTableHelper.col: item.,</v>
       </c>
       <c r="L21" t="str">
         <f t="shared" si="5"/>
-        <v>: map[ReceiptsTableHelper.col],</v>
+        <v>: map[NarrowEventsTableHelper.col],</v>
       </c>
       <c r="M21" t="str">
         <f t="shared" si="9"/>

</xml_diff>